<commit_message>
docs & core: update README, sync Ngrok badges & align system features
</commit_message>
<xml_diff>
--- a/Sales_Inventory.xlsx
+++ b/Sales_Inventory.xlsx
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J68"/>
+  <dimension ref="A1:J76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -590,7 +590,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -672,7 +672,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -713,7 +713,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -754,7 +754,7 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -795,7 +795,7 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -836,7 +836,7 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -877,7 +877,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -918,7 +918,7 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -959,7 +959,7 @@
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -1000,7 +1000,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1082,7 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -1123,7 +1123,7 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -1164,7 +1164,7 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -1205,7 +1205,7 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -1246,7 +1246,7 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -1287,7 +1287,7 @@
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -1328,7 +1328,7 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -1369,7 +1369,7 @@
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -1410,7 +1410,7 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -1451,7 +1451,7 @@
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -1492,7 +1492,7 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -1615,7 +1615,7 @@
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -1656,7 +1656,7 @@
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -1697,7 +1697,7 @@
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -1738,7 +1738,7 @@
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -1779,7 +1779,7 @@
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -1861,7 +1861,7 @@
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -1902,7 +1902,7 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -1943,7 +1943,7 @@
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -1984,7 +1984,7 @@
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -2025,7 +2025,7 @@
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -2066,7 +2066,7 @@
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -2107,7 +2107,7 @@
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -2148,7 +2148,7 @@
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -2189,7 +2189,7 @@
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -2230,7 +2230,7 @@
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -2271,7 +2271,7 @@
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -2312,7 +2312,7 @@
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -2353,7 +2353,7 @@
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -2394,7 +2394,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -2435,7 +2435,7 @@
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -2517,7 +2517,7 @@
       </c>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -2599,7 +2599,7 @@
       </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -2640,7 +2640,7 @@
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -2681,7 +2681,7 @@
       </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -2722,7 +2722,7 @@
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -2763,7 +2763,7 @@
       </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -2804,7 +2804,7 @@
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -2845,7 +2845,7 @@
       </c>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -2886,7 +2886,7 @@
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -2927,7 +2927,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -2968,7 +2968,7 @@
       </c>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -3009,7 +3009,7 @@
       </c>
       <c r="J61" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -3050,7 +3050,7 @@
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -3091,7 +3091,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -3132,7 +3132,7 @@
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -3173,7 +3173,7 @@
       </c>
       <c r="J65" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -3214,7 +3214,7 @@
       </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
@@ -3255,40 +3255,368 @@
       </c>
       <c r="J67" s="2" t="inlineStr">
         <is>
-          <t>Direct Sale</t>
+          <t>Sale</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="6" t="inlineStr">
+      <c r="A68" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>DE26002N</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E68" s="4" t="n">
+        <v>343.8</v>
+      </c>
+      <c r="F68" s="4">
+        <f>D68*E68</f>
+        <v/>
+      </c>
+      <c r="G68" s="4" t="n">
+        <v>235</v>
+      </c>
+      <c r="H68" s="4">
+        <f>F68-G68</f>
+        <v/>
+      </c>
+      <c r="I68" s="5">
+        <f>IF(F68&gt;0, H68/F68, 0)</f>
+        <v/>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>DE26050B</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E69" s="4" t="n">
+        <v>336.84</v>
+      </c>
+      <c r="F69" s="4">
+        <f>D69*E69</f>
+        <v/>
+      </c>
+      <c r="G69" s="4" t="n">
+        <v>235</v>
+      </c>
+      <c r="H69" s="4">
+        <f>F69-G69</f>
+        <v/>
+      </c>
+      <c r="I69" s="5">
+        <f>IF(F69&gt;0, H69/F69, 0)</f>
+        <v/>
+      </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>DE26002R</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E70" s="4" t="n">
+        <v>366.3</v>
+      </c>
+      <c r="F70" s="4">
+        <f>D70*E70</f>
+        <v/>
+      </c>
+      <c r="G70" s="4" t="n">
+        <v>235</v>
+      </c>
+      <c r="H70" s="4">
+        <f>F70-G70</f>
+        <v/>
+      </c>
+      <c r="I70" s="5">
+        <f>IF(F70&gt;0, H70/F70, 0)</f>
+        <v/>
+      </c>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>DE26002R</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E71" s="4" t="n">
+        <v>333.76</v>
+      </c>
+      <c r="F71" s="4">
+        <f>D71*E71</f>
+        <v/>
+      </c>
+      <c r="G71" s="4" t="n">
+        <v>235</v>
+      </c>
+      <c r="H71" s="4">
+        <f>F71-G71</f>
+        <v/>
+      </c>
+      <c r="I71" s="5">
+        <f>IF(F71&gt;0, H71/F71, 0)</f>
+        <v/>
+      </c>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>DE26009G</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E72" s="4" t="n">
+        <v>306.01</v>
+      </c>
+      <c r="F72" s="4">
+        <f>D72*E72</f>
+        <v/>
+      </c>
+      <c r="G72" s="4" t="n">
+        <v>225</v>
+      </c>
+      <c r="H72" s="4">
+        <f>F72-G72</f>
+        <v/>
+      </c>
+      <c r="I72" s="5">
+        <f>IF(F72&gt;0, H72/F72, 0)</f>
+        <v/>
+      </c>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>DE26050B</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E73" s="4" t="n">
+        <v>338.08</v>
+      </c>
+      <c r="F73" s="4">
+        <f>D73*E73</f>
+        <v/>
+      </c>
+      <c r="G73" s="4" t="n">
+        <v>235</v>
+      </c>
+      <c r="H73" s="4">
+        <f>F73-G73</f>
+        <v/>
+      </c>
+      <c r="I73" s="5">
+        <f>IF(F73&gt;0, H73/F73, 0)</f>
+        <v/>
+      </c>
+      <c r="J73" s="2" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>DE26077R</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E74" s="4" t="n">
+        <v>317.57</v>
+      </c>
+      <c r="F74" s="4">
+        <f>D74*E74</f>
+        <v/>
+      </c>
+      <c r="G74" s="4" t="n">
+        <v>220</v>
+      </c>
+      <c r="H74" s="4">
+        <f>F74-G74</f>
+        <v/>
+      </c>
+      <c r="I74" s="5">
+        <f>IF(F74&gt;0, H74/F74, 0)</f>
+        <v/>
+      </c>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>DE26081M</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E75" s="4" t="n">
+        <v>315.67</v>
+      </c>
+      <c r="F75" s="4">
+        <f>D75*E75</f>
+        <v/>
+      </c>
+      <c r="G75" s="4" t="n">
+        <v>235</v>
+      </c>
+      <c r="H75" s="4">
+        <f>F75-G75</f>
+        <v/>
+      </c>
+      <c r="I75" s="5">
+        <f>IF(F75&gt;0, H75/F75, 0)</f>
+        <v/>
+      </c>
+      <c r="J75" s="2" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="inlineStr">
         <is>
           <t>Total Summary</t>
         </is>
       </c>
-      <c r="B68" s="6" t="inlineStr"/>
-      <c r="C68" s="6" t="inlineStr"/>
-      <c r="D68" s="7">
-        <f>SUM(D2:D67)</f>
-        <v/>
-      </c>
-      <c r="E68" s="6" t="inlineStr"/>
-      <c r="F68" s="8">
-        <f>SUM(F2:F67)</f>
-        <v/>
-      </c>
-      <c r="G68" s="8">
-        <f>SUM(G2:G67)</f>
-        <v/>
-      </c>
-      <c r="H68" s="8">
-        <f>SUM(H2:H67)</f>
-        <v/>
-      </c>
-      <c r="I68" s="9">
-        <f>IF(F68&gt;0, H68/F68, 0)</f>
-        <v/>
-      </c>
-      <c r="J68" s="6" t="inlineStr"/>
+      <c r="B76" s="6" t="inlineStr"/>
+      <c r="C76" s="6" t="inlineStr"/>
+      <c r="D76" s="7">
+        <f>SUM(D2:D75)</f>
+        <v/>
+      </c>
+      <c r="E76" s="6" t="inlineStr"/>
+      <c r="F76" s="8">
+        <f>SUM(F2:F75)</f>
+        <v/>
+      </c>
+      <c r="G76" s="8">
+        <f>SUM(G2:G75)</f>
+        <v/>
+      </c>
+      <c r="H76" s="8">
+        <f>SUM(H2:H75)</f>
+        <v/>
+      </c>
+      <c r="I76" s="9">
+        <f>IF(F76&gt;0, H76/F76, 0)</f>
+        <v/>
+      </c>
+      <c r="J76" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3584,7 +3912,7 @@
         <v>8</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D7" s="3" t="n">
         <v>0</v>
@@ -3607,7 +3935,7 @@
         <v/>
       </c>
       <c r="J7" s="4" t="n">
-        <v>102.09</v>
+        <v>210.89</v>
       </c>
       <c r="K7" s="2">
         <f>IF(G7&gt;10, "In Stock", IF(G7&gt;0, "Low Stock", IF(G7=0, "Out of Stock", "Over Sold")))</f>
@@ -3624,7 +3952,7 @@
         <v>11</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>0</v>
@@ -3647,7 +3975,7 @@
         <v/>
       </c>
       <c r="J8" s="4" t="n">
-        <v>314.13</v>
+        <v>544.1900000000001</v>
       </c>
       <c r="K8" s="2">
         <f>IF(G8&gt;10, "In Stock", IF(G8&gt;0, "Low Stock", IF(G8=0, "Out of Stock", "Over Sold")))</f>
@@ -4344,7 +4672,7 @@
         <v>12</v>
       </c>
       <c r="C26" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D26" s="3" t="n">
         <v>0</v>
@@ -4367,7 +4695,7 @@
         <v/>
       </c>
       <c r="J26" s="4" t="n">
-        <v>284.14</v>
+        <v>365.15</v>
       </c>
       <c r="K26" s="2">
         <f>IF(G26&gt;10, "In Stock", IF(G26&gt;0, "Low Stock", IF(G26=0, "Out of Stock", "Over Sold")))</f>
@@ -4664,7 +4992,7 @@
         <v>10</v>
       </c>
       <c r="C34" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D34" s="3" t="n">
         <v>0</v>
@@ -4687,7 +5015,7 @@
         <v/>
       </c>
       <c r="J34" s="4" t="n">
-        <v>0</v>
+        <v>204.92</v>
       </c>
       <c r="K34" s="2">
         <f>IF(G34&gt;10, "In Stock", IF(G34&gt;0, "Low Stock", IF(G34=0, "Out of Stock", "Over Sold")))</f>
@@ -4824,7 +5152,7 @@
         <v>12</v>
       </c>
       <c r="C38" s="3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D38" s="3" t="n">
         <v>0</v>
@@ -4847,7 +5175,7 @@
         <v/>
       </c>
       <c r="J38" s="4" t="n">
-        <v>488.18</v>
+        <v>585.75</v>
       </c>
       <c r="K38" s="2">
         <f>IF(G38&gt;10, "In Stock", IF(G38&gt;0, "Low Stock", IF(G38=0, "Out of Stock", "Over Sold")))</f>
@@ -4867,10 +5195,10 @@
         <v>6</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F39" s="3" t="n">
         <v>0</v>
@@ -4904,7 +5232,7 @@
         <v>10</v>
       </c>
       <c r="C40" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D40" s="3" t="n">
         <v>0</v>
@@ -4927,7 +5255,7 @@
         <v/>
       </c>
       <c r="J40" s="4" t="n">
-        <v>0</v>
+        <v>80.67</v>
       </c>
       <c r="K40" s="2">
         <f>IF(G40&gt;10, "In Stock", IF(G40&gt;0, "Low Stock", IF(G40=0, "Out of Stock", "Over Sold")))</f>
@@ -5548,10 +5876,14 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>In Transit</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr"/>
+          <t>Received</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr">
         <is>
@@ -5652,7 +5984,7 @@
     <col width="19" customWidth="1" min="6" max="6"/>
     <col width="37" customWidth="1" min="7" max="7"/>
     <col width="48" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
     <col width="17" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
     <col width="34" customWidth="1" min="12" max="12"/>
@@ -5975,10 +6307,14 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>In Transit</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr"/>
+          <t>Received</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr">
         <is>
@@ -6257,7 +6593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -6737,17 +7073,49 @@
       <c r="D29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="inlineStr">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Meesho Ads</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="n">
+        <v>332.49</v>
+      </c>
+      <c r="D30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Meesho Ads</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="n">
+        <v>316.36</v>
+      </c>
+      <c r="D31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>Total Summary</t>
         </is>
       </c>
-      <c r="B30" s="6" t="inlineStr"/>
-      <c r="C30" s="8">
-        <f>SUM(C2:C29)</f>
-        <v/>
-      </c>
-      <c r="D30" s="6" t="inlineStr"/>
+      <c r="B32" s="6" t="inlineStr"/>
+      <c r="C32" s="8">
+        <f>SUM(C2:C31)</f>
+        <v/>
+      </c>
+      <c r="D32" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6760,12 +7128,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="23" customWidth="1" min="5" max="5"/>
   </cols>
@@ -7029,18 +7397,39 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Credited (+)</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>269.85</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>-112541.37</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>Total Summary</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr"/>
-      <c r="C13" s="6" t="inlineStr"/>
-      <c r="D13" s="8">
-        <f>SUM(D2:D12)</f>
-        <v/>
-      </c>
-      <c r="E13" s="6" t="inlineStr"/>
+      <c r="B14" s="6" t="inlineStr"/>
+      <c r="C14" s="6" t="inlineStr"/>
+      <c r="D14" s="8">
+        <f>SUM(D2:D13)</f>
+        <v/>
+      </c>
+      <c r="E14" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7053,7 +7442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -7724,33 +8113,87 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C25" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D25" s="4" t="n">
+        <v>1046.94</v>
+      </c>
+      <c r="E25" s="4" t="n">
+        <v>705</v>
+      </c>
+      <c r="F25" s="4">
+        <f>D25-E25</f>
+        <v/>
+      </c>
+      <c r="G25" s="5">
+        <f>IF(D25&gt;0, F25/D25, 0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C26" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D26" s="4" t="n">
+        <v>1611.09</v>
+      </c>
+      <c r="E26" s="4" t="n">
+        <v>1150</v>
+      </c>
+      <c r="F26" s="4">
+        <f>D26-E26</f>
+        <v/>
+      </c>
+      <c r="G26" s="5">
+        <f>IF(D26&gt;0, F26/D26, 0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
         <is>
           <t>Total Summary</t>
         </is>
       </c>
-      <c r="B25" s="7">
-        <f>SUM(B2:B24)</f>
-        <v/>
-      </c>
-      <c r="C25" s="7">
-        <f>SUM(C2:C24)</f>
-        <v/>
-      </c>
-      <c r="D25" s="8">
-        <f>SUM(D2:D24)</f>
-        <v/>
-      </c>
-      <c r="E25" s="8">
-        <f>SUM(E2:E24)</f>
-        <v/>
-      </c>
-      <c r="F25" s="8">
-        <f>SUM(F2:F24)</f>
-        <v/>
-      </c>
-      <c r="G25" s="9">
-        <f>IF(D25&gt;0, F25/D25, 0)</f>
+      <c r="B27" s="7">
+        <f>SUM(B2:B26)</f>
+        <v/>
+      </c>
+      <c r="C27" s="7">
+        <f>SUM(C2:C26)</f>
+        <v/>
+      </c>
+      <c r="D27" s="8">
+        <f>SUM(D2:D26)</f>
+        <v/>
+      </c>
+      <c r="E27" s="8">
+        <f>SUM(E2:E26)</f>
+        <v/>
+      </c>
+      <c r="F27" s="8">
+        <f>SUM(F2:F26)</f>
+        <v/>
+      </c>
+      <c r="G27" s="9">
+        <f>IF(D27&gt;0, F27/D27, 0)</f>
         <v/>
       </c>
     </row>
@@ -7765,7 +8208,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -8193,18 +8636,54 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Meesho Ads</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="n">
+        <v>332.49</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Meesho Ads</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="n">
+        <v>316.36</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
         <is>
           <t>Total Summary</t>
         </is>
       </c>
-      <c r="B24" s="7">
-        <f>SUM(B2:B23)</f>
-        <v/>
-      </c>
-      <c r="C24" s="6" t="inlineStr"/>
-      <c r="D24" s="8">
-        <f>SUM(D2:D23)</f>
+      <c r="B26" s="7">
+        <f>SUM(B2:B25)</f>
+        <v/>
+      </c>
+      <c r="C26" s="6" t="inlineStr"/>
+      <c r="D26" s="8">
+        <f>SUM(D2:D25)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: integrate Barcode Master, Meesho Catalog, live formula engine, and reverse-engineered barcode generator
</commit_message>
<xml_diff>
--- a/Sales_Inventory.xlsx
+++ b/Sales_Inventory.xlsx
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J76"/>
+  <dimension ref="A1:J96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -3588,35 +3588,855 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="6" t="inlineStr">
+      <c r="A76" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>DE26002R</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E76" s="4" t="n">
+        <v>366.84</v>
+      </c>
+      <c r="F76" s="4">
+        <f>D76*E76</f>
+        <v/>
+      </c>
+      <c r="G76" s="4" t="n">
+        <v>470</v>
+      </c>
+      <c r="H76" s="4">
+        <f>F76-G76</f>
+        <v/>
+      </c>
+      <c r="I76" s="5">
+        <f>IF(F76&gt;0, H76/F76, 0)</f>
+        <v/>
+      </c>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>DE26003W</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E77" s="4" t="n">
+        <v>326</v>
+      </c>
+      <c r="F77" s="4">
+        <f>D77*E77</f>
+        <v/>
+      </c>
+      <c r="G77" s="4" t="n">
+        <v>438</v>
+      </c>
+      <c r="H77" s="4">
+        <f>F77-G77</f>
+        <v/>
+      </c>
+      <c r="I77" s="5">
+        <f>IF(F77&gt;0, H77/F77, 0)</f>
+        <v/>
+      </c>
+      <c r="J77" s="2" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>DE26006R</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E78" s="4" t="n">
+        <v>337.71</v>
+      </c>
+      <c r="F78" s="4">
+        <f>D78*E78</f>
+        <v/>
+      </c>
+      <c r="G78" s="4" t="n">
+        <v>235</v>
+      </c>
+      <c r="H78" s="4">
+        <f>F78-G78</f>
+        <v/>
+      </c>
+      <c r="I78" s="5">
+        <f>IF(F78&gt;0, H78/F78, 0)</f>
+        <v/>
+      </c>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>DE26009B</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E79" s="4" t="n">
+        <v>328.01</v>
+      </c>
+      <c r="F79" s="4">
+        <f>D79*E79</f>
+        <v/>
+      </c>
+      <c r="G79" s="4" t="n">
+        <v>225</v>
+      </c>
+      <c r="H79" s="4">
+        <f>F79-G79</f>
+        <v/>
+      </c>
+      <c r="I79" s="5">
+        <f>IF(F79&gt;0, H79/F79, 0)</f>
+        <v/>
+      </c>
+      <c r="J79" s="2" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>DE26009Y</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E80" s="4" t="n">
+        <v>294.62</v>
+      </c>
+      <c r="F80" s="4">
+        <f>D80*E80</f>
+        <v/>
+      </c>
+      <c r="G80" s="4" t="n">
+        <v>225</v>
+      </c>
+      <c r="H80" s="4">
+        <f>F80-G80</f>
+        <v/>
+      </c>
+      <c r="I80" s="5">
+        <f>IF(F80&gt;0, H80/F80, 0)</f>
+        <v/>
+      </c>
+      <c r="J80" s="2" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>DE26077R</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E81" s="4" t="n">
+        <v>286.25</v>
+      </c>
+      <c r="F81" s="4">
+        <f>D81*E81</f>
+        <v/>
+      </c>
+      <c r="G81" s="4" t="n">
+        <v>220</v>
+      </c>
+      <c r="H81" s="4">
+        <f>F81-G81</f>
+        <v/>
+      </c>
+      <c r="I81" s="5">
+        <f>IF(F81&gt;0, H81/F81, 0)</f>
+        <v/>
+      </c>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>DE26077Y</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E82" s="4" t="n">
+        <v>287.22</v>
+      </c>
+      <c r="F82" s="4">
+        <f>D82*E82</f>
+        <v/>
+      </c>
+      <c r="G82" s="4" t="n">
+        <v>220</v>
+      </c>
+      <c r="H82" s="4">
+        <f>F82-G82</f>
+        <v/>
+      </c>
+      <c r="I82" s="5">
+        <f>IF(F82&gt;0, H82/F82, 0)</f>
+        <v/>
+      </c>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>DE26002N</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E83" s="4" t="n">
+        <v>365.53</v>
+      </c>
+      <c r="F83" s="4">
+        <f>D83*E83</f>
+        <v/>
+      </c>
+      <c r="G83" s="4" t="n">
+        <v>235</v>
+      </c>
+      <c r="H83" s="4">
+        <f>F83-G83</f>
+        <v/>
+      </c>
+      <c r="I83" s="5">
+        <f>IF(F83&gt;0, H83/F83, 0)</f>
+        <v/>
+      </c>
+      <c r="J83" s="2" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>DE26007N</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E84" s="4" t="n">
+        <v>302.73</v>
+      </c>
+      <c r="F84" s="4">
+        <f>D84*E84</f>
+        <v/>
+      </c>
+      <c r="G84" s="4" t="n">
+        <v>235</v>
+      </c>
+      <c r="H84" s="4">
+        <f>F84-G84</f>
+        <v/>
+      </c>
+      <c r="I84" s="5">
+        <f>IF(F84&gt;0, H84/F84, 0)</f>
+        <v/>
+      </c>
+      <c r="J84" s="2" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>DE26009G</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E85" s="4" t="n">
+        <v>295.66</v>
+      </c>
+      <c r="F85" s="4">
+        <f>D85*E85</f>
+        <v/>
+      </c>
+      <c r="G85" s="4" t="n">
+        <v>225</v>
+      </c>
+      <c r="H85" s="4">
+        <f>F85-G85</f>
+        <v/>
+      </c>
+      <c r="I85" s="5">
+        <f>IF(F85&gt;0, H85/F85, 0)</f>
+        <v/>
+      </c>
+      <c r="J85" s="2" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>DE26077N</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E86" s="4" t="n">
+        <v>283.69</v>
+      </c>
+      <c r="F86" s="4">
+        <f>D86*E86</f>
+        <v/>
+      </c>
+      <c r="G86" s="4" t="n">
+        <v>220</v>
+      </c>
+      <c r="H86" s="4">
+        <f>F86-G86</f>
+        <v/>
+      </c>
+      <c r="I86" s="5">
+        <f>IF(F86&gt;0, H86/F86, 0)</f>
+        <v/>
+      </c>
+      <c r="J86" s="2" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>DE26005N</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E87" s="4" t="n">
+        <v>304.28</v>
+      </c>
+      <c r="F87" s="4">
+        <f>D87*E87</f>
+        <v/>
+      </c>
+      <c r="G87" s="4" t="n">
+        <v>235</v>
+      </c>
+      <c r="H87" s="4">
+        <f>F87-G87</f>
+        <v/>
+      </c>
+      <c r="I87" s="5">
+        <f>IF(F87&gt;0, H87/F87, 0)</f>
+        <v/>
+      </c>
+      <c r="J87" s="2" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>DE26077R</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E88" s="4" t="n">
+        <v>318.53</v>
+      </c>
+      <c r="F88" s="4">
+        <f>D88*E88</f>
+        <v/>
+      </c>
+      <c r="G88" s="4" t="n">
+        <v>220</v>
+      </c>
+      <c r="H88" s="4">
+        <f>F88-G88</f>
+        <v/>
+      </c>
+      <c r="I88" s="5">
+        <f>IF(F88&gt;0, H88/F88, 0)</f>
+        <v/>
+      </c>
+      <c r="J88" s="2" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>DE26016R</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E89" s="4" t="n">
+        <v>292.51</v>
+      </c>
+      <c r="F89" s="4">
+        <f>D89*E89</f>
+        <v/>
+      </c>
+      <c r="G89" s="4" t="n">
+        <v>235</v>
+      </c>
+      <c r="H89" s="4">
+        <f>F89-G89</f>
+        <v/>
+      </c>
+      <c r="I89" s="5">
+        <f>IF(F89&gt;0, H89/F89, 0)</f>
+        <v/>
+      </c>
+      <c r="J89" s="2" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>DE26077Y</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E90" s="4" t="n">
+        <v>297.2</v>
+      </c>
+      <c r="F90" s="4">
+        <f>D90*E90</f>
+        <v/>
+      </c>
+      <c r="G90" s="4" t="n">
+        <v>220</v>
+      </c>
+      <c r="H90" s="4">
+        <f>F90-G90</f>
+        <v/>
+      </c>
+      <c r="I90" s="5">
+        <f>IF(F90&gt;0, H90/F90, 0)</f>
+        <v/>
+      </c>
+      <c r="J90" s="2" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>DE26077R</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E91" s="4" t="n">
+        <v>297.32</v>
+      </c>
+      <c r="F91" s="4">
+        <f>D91*E91</f>
+        <v/>
+      </c>
+      <c r="G91" s="4" t="n">
+        <v>440</v>
+      </c>
+      <c r="H91" s="4">
+        <f>F91-G91</f>
+        <v/>
+      </c>
+      <c r="I91" s="5">
+        <f>IF(F91&gt;0, H91/F91, 0)</f>
+        <v/>
+      </c>
+      <c r="J91" s="2" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>DE26002R</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E92" s="4" t="n">
+        <v>366.43</v>
+      </c>
+      <c r="F92" s="4">
+        <f>D92*E92</f>
+        <v/>
+      </c>
+      <c r="G92" s="4" t="n">
+        <v>235</v>
+      </c>
+      <c r="H92" s="4">
+        <f>F92-G92</f>
+        <v/>
+      </c>
+      <c r="I92" s="5">
+        <f>IF(F92&gt;0, H92/F92, 0)</f>
+        <v/>
+      </c>
+      <c r="J92" s="2" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>DE26009B</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E93" s="4" t="n">
+        <v>305.08</v>
+      </c>
+      <c r="F93" s="4">
+        <f>D93*E93</f>
+        <v/>
+      </c>
+      <c r="G93" s="4" t="n">
+        <v>225</v>
+      </c>
+      <c r="H93" s="4">
+        <f>F93-G93</f>
+        <v/>
+      </c>
+      <c r="I93" s="5">
+        <f>IF(F93&gt;0, H93/F93, 0)</f>
+        <v/>
+      </c>
+      <c r="J93" s="2" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>DE26030B</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E94" s="4" t="n">
+        <v>291.97</v>
+      </c>
+      <c r="F94" s="4">
+        <f>D94*E94</f>
+        <v/>
+      </c>
+      <c r="G94" s="4" t="n">
+        <v>205</v>
+      </c>
+      <c r="H94" s="4">
+        <f>F94-G94</f>
+        <v/>
+      </c>
+      <c r="I94" s="5">
+        <f>IF(F94&gt;0, H94/F94, 0)</f>
+        <v/>
+      </c>
+      <c r="J94" s="2" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>DE26009G</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E95" s="4" t="n">
+        <v>305.27</v>
+      </c>
+      <c r="F95" s="4">
+        <f>D95*E95</f>
+        <v/>
+      </c>
+      <c r="G95" s="4" t="n">
+        <v>225</v>
+      </c>
+      <c r="H95" s="4">
+        <f>F95-G95</f>
+        <v/>
+      </c>
+      <c r="I95" s="5">
+        <f>IF(F95&gt;0, H95/F95, 0)</f>
+        <v/>
+      </c>
+      <c r="J95" s="2" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="6" t="inlineStr">
         <is>
           <t>Total Summary</t>
         </is>
       </c>
-      <c r="B76" s="6" t="inlineStr"/>
-      <c r="C76" s="6" t="inlineStr"/>
-      <c r="D76" s="7">
-        <f>SUM(D2:D75)</f>
-        <v/>
-      </c>
-      <c r="E76" s="6" t="inlineStr"/>
-      <c r="F76" s="8">
-        <f>SUM(F2:F75)</f>
-        <v/>
-      </c>
-      <c r="G76" s="8">
-        <f>SUM(G2:G75)</f>
-        <v/>
-      </c>
-      <c r="H76" s="8">
-        <f>SUM(H2:H75)</f>
-        <v/>
-      </c>
-      <c r="I76" s="9">
-        <f>IF(F76&gt;0, H76/F76, 0)</f>
-        <v/>
-      </c>
-      <c r="J76" s="6" t="inlineStr"/>
+      <c r="B96" s="6" t="inlineStr"/>
+      <c r="C96" s="6" t="inlineStr"/>
+      <c r="D96" s="7">
+        <f>SUM(D2:D95)</f>
+        <v/>
+      </c>
+      <c r="E96" s="6" t="inlineStr"/>
+      <c r="F96" s="8">
+        <f>SUM(F2:F95)</f>
+        <v/>
+      </c>
+      <c r="G96" s="8">
+        <f>SUM(G2:G95)</f>
+        <v/>
+      </c>
+      <c r="H96" s="8">
+        <f>SUM(H2:H95)</f>
+        <v/>
+      </c>
+      <c r="I96" s="9">
+        <f>IF(F96&gt;0, H96/F96, 0)</f>
+        <v/>
+      </c>
+      <c r="J96" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3912,7 +4732,7 @@
         <v>8</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D7" s="3" t="n">
         <v>0</v>
@@ -3935,7 +4755,7 @@
         <v/>
       </c>
       <c r="J7" s="4" t="n">
-        <v>210.89</v>
+        <v>341.42</v>
       </c>
       <c r="K7" s="2">
         <f>IF(G7&gt;10, "In Stock", IF(G7&gt;0, "Low Stock", IF(G7=0, "Out of Stock", "Over Sold")))</f>
@@ -3952,13 +4772,13 @@
         <v>11</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>0</v>
@@ -3975,7 +4795,7 @@
         <v/>
       </c>
       <c r="J8" s="4" t="n">
-        <v>544.1900000000001</v>
+        <v>939.3000000000001</v>
       </c>
       <c r="K8" s="2">
         <f>IF(G8&gt;10, "In Stock", IF(G8&gt;0, "Low Stock", IF(G8=0, "Out of Stock", "Over Sold")))</f>
@@ -4032,7 +4852,7 @@
         <v>30</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D10" s="3" t="n">
         <v>0</v>
@@ -4055,7 +4875,7 @@
         <v/>
       </c>
       <c r="J10" s="4" t="n">
-        <v>2185.64</v>
+        <v>2399.64</v>
       </c>
       <c r="K10" s="2">
         <f>IF(G10&gt;10, "In Stock", IF(G10&gt;0, "Low Stock", IF(G10=0, "Out of Stock", "Over Sold")))</f>
@@ -4232,7 +5052,7 @@
         <v>10</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D15" s="3" t="n">
         <v>0</v>
@@ -4255,7 +5075,7 @@
         <v/>
       </c>
       <c r="J15" s="4" t="n">
-        <v>36.06</v>
+        <v>105.34</v>
       </c>
       <c r="K15" s="2">
         <f>IF(G15&gt;10, "In Stock", IF(G15&gt;0, "Low Stock", IF(G15=0, "Out of Stock", "Over Sold")))</f>
@@ -4352,7 +5172,7 @@
         <v>10</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D18" s="3" t="n">
         <v>0</v>
@@ -4375,7 +5195,7 @@
         <v/>
       </c>
       <c r="J18" s="4" t="n">
-        <v>400.68</v>
+        <v>503.39</v>
       </c>
       <c r="K18" s="2">
         <f>IF(G18&gt;10, "In Stock", IF(G18&gt;0, "Low Stock", IF(G18=0, "Out of Stock", "Over Sold")))</f>
@@ -4432,7 +5252,7 @@
         <v>7</v>
       </c>
       <c r="C20" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D20" s="3" t="n">
         <v>0</v>
@@ -4455,7 +5275,7 @@
         <v/>
       </c>
       <c r="J20" s="4" t="n">
-        <v>181.53</v>
+        <v>249.26</v>
       </c>
       <c r="K20" s="2">
         <f>IF(G20&gt;10, "In Stock", IF(G20&gt;0, "Low Stock", IF(G20=0, "Out of Stock", "Over Sold")))</f>
@@ -4632,7 +5452,7 @@
         <v>13</v>
       </c>
       <c r="C25" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D25" s="3" t="n">
         <v>0</v>
@@ -4655,7 +5475,7 @@
         <v/>
       </c>
       <c r="J25" s="4" t="n">
-        <v>0</v>
+        <v>183.09</v>
       </c>
       <c r="K25" s="2">
         <f>IF(G25&gt;10, "In Stock", IF(G25&gt;0, "Low Stock", IF(G25=0, "Out of Stock", "Over Sold")))</f>
@@ -4672,7 +5492,7 @@
         <v>12</v>
       </c>
       <c r="C26" s="3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D26" s="3" t="n">
         <v>0</v>
@@ -4695,7 +5515,7 @@
         <v/>
       </c>
       <c r="J26" s="4" t="n">
-        <v>365.15</v>
+        <v>516.08</v>
       </c>
       <c r="K26" s="2">
         <f>IF(G26&gt;10, "In Stock", IF(G26&gt;0, "Low Stock", IF(G26=0, "Out of Stock", "Over Sold")))</f>
@@ -4715,7 +5535,7 @@
         <v>1</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E27" s="3" t="n">
         <v>0</v>
@@ -4752,7 +5572,7 @@
         <v>13</v>
       </c>
       <c r="C28" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D28" s="3" t="n">
         <v>0</v>
@@ -4775,7 +5595,7 @@
         <v/>
       </c>
       <c r="J28" s="4" t="n">
-        <v>0</v>
+        <v>69.62</v>
       </c>
       <c r="K28" s="2">
         <f>IF(G28&gt;10, "In Stock", IF(G28&gt;0, "Low Stock", IF(G28=0, "Out of Stock", "Over Sold")))</f>
@@ -4832,7 +5652,7 @@
         <v>10</v>
       </c>
       <c r="C30" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D30" s="3" t="n">
         <v>0</v>
@@ -4855,7 +5675,7 @@
         <v/>
       </c>
       <c r="J30" s="4" t="n">
-        <v>0</v>
+        <v>57.51</v>
       </c>
       <c r="K30" s="2">
         <f>IF(G30&gt;10, "In Stock", IF(G30&gt;0, "Low Stock", IF(G30=0, "Out of Stock", "Over Sold")))</f>
@@ -4872,7 +5692,7 @@
         <v>10</v>
       </c>
       <c r="C31" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D31" s="3" t="n">
         <v>0</v>
@@ -4895,7 +5715,7 @@
         <v/>
       </c>
       <c r="J31" s="4" t="n">
-        <v>262.55</v>
+        <v>349.52</v>
       </c>
       <c r="K31" s="2">
         <f>IF(G31&gt;10, "In Stock", IF(G31&gt;0, "Low Stock", IF(G31=0, "Out of Stock", "Over Sold")))</f>
@@ -5112,7 +5932,7 @@
         <v>6</v>
       </c>
       <c r="C37" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D37" s="3" t="n">
         <v>0</v>
@@ -5135,7 +5955,7 @@
         <v/>
       </c>
       <c r="J37" s="4" t="n">
-        <v>401.56</v>
+        <v>465.25</v>
       </c>
       <c r="K37" s="2">
         <f>IF(G37&gt;10, "In Stock", IF(G37&gt;0, "Low Stock", IF(G37=0, "Out of Stock", "Over Sold")))</f>
@@ -5152,7 +5972,7 @@
         <v>12</v>
       </c>
       <c r="C38" s="3" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D38" s="3" t="n">
         <v>0</v>
@@ -5175,7 +5995,7 @@
         <v/>
       </c>
       <c r="J38" s="4" t="n">
-        <v>585.75</v>
+        <v>905.17</v>
       </c>
       <c r="K38" s="2">
         <f>IF(G38&gt;10, "In Stock", IF(G38&gt;0, "Low Stock", IF(G38=0, "Out of Stock", "Over Sold")))</f>
@@ -5192,13 +6012,13 @@
         <v>12</v>
       </c>
       <c r="C39" s="3" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F39" s="3" t="n">
         <v>0</v>
@@ -5215,7 +6035,7 @@
         <v/>
       </c>
       <c r="J39" s="4" t="n">
-        <v>463.42</v>
+        <v>607.84</v>
       </c>
       <c r="K39" s="2">
         <f>IF(G39&gt;10, "In Stock", IF(G39&gt;0, "Low Stock", IF(G39=0, "Out of Stock", "Over Sold")))</f>
@@ -5394,7 +6214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -5833,10 +6653,14 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>In Transit</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr"/>
+          <t>Received</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
       <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr">
         <is>
@@ -5936,31 +6760,121 @@
       <c r="L11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>RTO-011</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>DE26009P</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>302.1</v>
+      </c>
+      <c r="F12" s="4">
+        <f>D12*E12</f>
+        <v/>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>In Transit</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Valmo AWB-VL0085381962558</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>RTO-012</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>DE26002R</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>315.37</v>
+      </c>
+      <c r="F13" s="4">
+        <f>D13*E13</f>
+        <v/>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Received</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Delhivery AWB-1490841138769286</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>Total Summary</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr"/>
-      <c r="C12" s="6" t="inlineStr"/>
-      <c r="D12" s="7">
-        <f>SUM(D2:D11)</f>
-        <v/>
-      </c>
-      <c r="E12" s="6" t="inlineStr"/>
-      <c r="F12" s="8">
-        <f>SUM(F2:F11)</f>
-        <v/>
-      </c>
-      <c r="G12" s="8">
-        <f>SUM(G2:G11)</f>
-        <v/>
-      </c>
-      <c r="H12" s="6" t="inlineStr"/>
-      <c r="I12" s="6" t="inlineStr"/>
-      <c r="J12" s="6" t="inlineStr"/>
-      <c r="K12" s="6" t="inlineStr"/>
-      <c r="L12" s="6" t="inlineStr"/>
+      <c r="B14" s="6" t="inlineStr"/>
+      <c r="C14" s="6" t="inlineStr"/>
+      <c r="D14" s="7">
+        <f>SUM(D2:D13)</f>
+        <v/>
+      </c>
+      <c r="E14" s="6" t="inlineStr"/>
+      <c r="F14" s="8">
+        <f>SUM(F2:F13)</f>
+        <v/>
+      </c>
+      <c r="G14" s="8">
+        <f>SUM(G2:G13)</f>
+        <v/>
+      </c>
+      <c r="H14" s="6" t="inlineStr"/>
+      <c r="I14" s="6" t="inlineStr"/>
+      <c r="J14" s="6" t="inlineStr"/>
+      <c r="K14" s="6" t="inlineStr"/>
+      <c r="L14" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5973,7 +6887,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -5984,7 +6898,7 @@
     <col width="19" customWidth="1" min="6" max="6"/>
     <col width="37" customWidth="1" min="7" max="7"/>
     <col width="48" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
     <col width="17" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
     <col width="34" customWidth="1" min="12" max="12"/>
@@ -6324,32 +7238,179 @@
       <c r="M6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>CR-006</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>DE26006R</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>309.82</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>175</v>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Product's quality or performance is not good</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>In Transit</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Valmo AWB-VLR082916892869</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>CR-007</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>DE26002M</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>366.57</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>175</v>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Don't need the product anymore</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Found lower price elsewhere</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>In Transit</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Valmo AWB-VLR082918756063</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>CR-008</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>DE26002N</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>343.8</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>175</v>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Wrong size delivered</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>In Transit</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Shadowfax AWB-R2567239146FPL</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>Total Summary</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr"/>
-      <c r="C7" s="6" t="inlineStr"/>
-      <c r="D7" s="7">
-        <f>SUM(D2:D6)</f>
-        <v/>
-      </c>
-      <c r="E7" s="8">
-        <f>SUM(E2:E6)</f>
-        <v/>
-      </c>
-      <c r="F7" s="8">
-        <f>SUM(F2:F6)</f>
-        <v/>
-      </c>
-      <c r="G7" s="6" t="inlineStr"/>
-      <c r="H7" s="6" t="inlineStr"/>
-      <c r="I7" s="6" t="inlineStr"/>
-      <c r="J7" s="6" t="inlineStr"/>
-      <c r="K7" s="6" t="inlineStr"/>
-      <c r="L7" s="6" t="inlineStr"/>
-      <c r="M7" s="6" t="inlineStr"/>
+      <c r="B10" s="6" t="inlineStr"/>
+      <c r="C10" s="6" t="inlineStr"/>
+      <c r="D10" s="7">
+        <f>SUM(D2:D9)</f>
+        <v/>
+      </c>
+      <c r="E10" s="8">
+        <f>SUM(E2:E9)</f>
+        <v/>
+      </c>
+      <c r="F10" s="8">
+        <f>SUM(F2:F9)</f>
+        <v/>
+      </c>
+      <c r="G10" s="6" t="inlineStr"/>
+      <c r="H10" s="6" t="inlineStr"/>
+      <c r="I10" s="6" t="inlineStr"/>
+      <c r="J10" s="6" t="inlineStr"/>
+      <c r="K10" s="6" t="inlineStr"/>
+      <c r="L10" s="6" t="inlineStr"/>
+      <c r="M10" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6593,7 +7654,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -7105,17 +8166,49 @@
       <c r="D31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="inlineStr">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Meesho Ads</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="n">
+        <v>301.32</v>
+      </c>
+      <c r="D32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Meesho Ads</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="D33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
         <is>
           <t>Total Summary</t>
         </is>
       </c>
-      <c r="B32" s="6" t="inlineStr"/>
-      <c r="C32" s="8">
-        <f>SUM(C2:C31)</f>
-        <v/>
-      </c>
-      <c r="D32" s="6" t="inlineStr"/>
+      <c r="B34" s="6" t="inlineStr"/>
+      <c r="C34" s="8">
+        <f>SUM(C2:C33)</f>
+        <v/>
+      </c>
+      <c r="D34" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7128,7 +8221,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -7418,18 +8511,102 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Credited (+)</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>948.09</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>-111593.28</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Credited (+)</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>310.13</v>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>-111283.15</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Credited (+)</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>593.05</v>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>-110690.1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Credited (+)</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>1056.85</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>-109633.25</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>Total Summary</t>
         </is>
       </c>
-      <c r="B14" s="6" t="inlineStr"/>
-      <c r="C14" s="6" t="inlineStr"/>
-      <c r="D14" s="8">
-        <f>SUM(D2:D13)</f>
-        <v/>
-      </c>
-      <c r="E14" s="6" t="inlineStr"/>
+      <c r="B18" s="6" t="inlineStr"/>
+      <c r="C18" s="6" t="inlineStr"/>
+      <c r="D18" s="8">
+        <f>SUM(D2:D17)</f>
+        <v/>
+      </c>
+      <c r="E18" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7442,7 +8619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -8167,33 +9344,195 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="inlineStr">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C27" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D27" s="4" t="n">
+        <v>2051.4</v>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F27" s="4">
+        <f>D27-E27</f>
+        <v/>
+      </c>
+      <c r="G27" s="5">
+        <f>IF(D27&gt;0, F27/D27, 0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D28" s="4" t="n">
+        <v>868.09</v>
+      </c>
+      <c r="E28" s="4" t="n">
+        <v>665</v>
+      </c>
+      <c r="F28" s="4">
+        <f>D28-E28</f>
+        <v/>
+      </c>
+      <c r="G28" s="5">
+        <f>IF(D28&gt;0, F28/D28, 0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C29" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D29" s="4" t="n">
+        <v>1247.61</v>
+      </c>
+      <c r="E29" s="4" t="n">
+        <v>915</v>
+      </c>
+      <c r="F29" s="4">
+        <f>D29-E29</f>
+        <v/>
+      </c>
+      <c r="G29" s="5">
+        <f>IF(D29&gt;0, F29/D29, 0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C30" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D30" s="4" t="n">
+        <v>622.8099999999999</v>
+      </c>
+      <c r="E30" s="4" t="n">
+        <v>455</v>
+      </c>
+      <c r="F30" s="4">
+        <f>D30-E30</f>
+        <v/>
+      </c>
+      <c r="G30" s="5">
+        <f>IF(D30&gt;0, F30/D30, 0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C31" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D31" s="4" t="n">
+        <v>1184.35</v>
+      </c>
+      <c r="E31" s="4" t="n">
+        <v>895</v>
+      </c>
+      <c r="F31" s="4">
+        <f>D31-E31</f>
+        <v/>
+      </c>
+      <c r="G31" s="5">
+        <f>IF(D31&gt;0, F31/D31, 0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C32" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D32" s="4" t="n">
+        <v>1268.75</v>
+      </c>
+      <c r="E32" s="4" t="n">
+        <v>890</v>
+      </c>
+      <c r="F32" s="4">
+        <f>D32-E32</f>
+        <v/>
+      </c>
+      <c r="G32" s="5">
+        <f>IF(D32&gt;0, F32/D32, 0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
         <is>
           <t>Total Summary</t>
         </is>
       </c>
-      <c r="B27" s="7">
-        <f>SUM(B2:B26)</f>
-        <v/>
-      </c>
-      <c r="C27" s="7">
-        <f>SUM(C2:C26)</f>
-        <v/>
-      </c>
-      <c r="D27" s="8">
-        <f>SUM(D2:D26)</f>
-        <v/>
-      </c>
-      <c r="E27" s="8">
-        <f>SUM(E2:E26)</f>
-        <v/>
-      </c>
-      <c r="F27" s="8">
-        <f>SUM(F2:F26)</f>
-        <v/>
-      </c>
-      <c r="G27" s="9">
-        <f>IF(D27&gt;0, F27/D27, 0)</f>
+      <c r="B33" s="7">
+        <f>SUM(B2:B32)</f>
+        <v/>
+      </c>
+      <c r="C33" s="7">
+        <f>SUM(C2:C32)</f>
+        <v/>
+      </c>
+      <c r="D33" s="8">
+        <f>SUM(D2:D32)</f>
+        <v/>
+      </c>
+      <c r="E33" s="8">
+        <f>SUM(E2:E32)</f>
+        <v/>
+      </c>
+      <c r="F33" s="8">
+        <f>SUM(F2:F32)</f>
+        <v/>
+      </c>
+      <c r="G33" s="9">
+        <f>IF(D33&gt;0, F33/D33, 0)</f>
         <v/>
       </c>
     </row>
@@ -8208,7 +9547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -8672,18 +10011,54 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Meesho Ads</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="n">
+        <v>301.32</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Meesho Ads</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
         <is>
           <t>Total Summary</t>
         </is>
       </c>
-      <c r="B26" s="7">
-        <f>SUM(B2:B25)</f>
-        <v/>
-      </c>
-      <c r="C26" s="6" t="inlineStr"/>
-      <c r="D26" s="8">
-        <f>SUM(D2:D25)</f>
+      <c r="B28" s="7">
+        <f>SUM(B2:B27)</f>
+        <v/>
+      </c>
+      <c r="C28" s="6" t="inlineStr"/>
+      <c r="D28" s="8">
+        <f>SUM(D2:D27)</f>
         <v/>
       </c>
     </row>

</xml_diff>